<commit_message>
Fix importante. Alineacion de variables Pantalla	Cambios SCR-000	12 renombres (qd_seguro→qd_productoSFC, qd_motivo→qd_motivoSFC, qd_detalle→qd_textoQueja, qd_pais→qd_codigoPais, qd_ciudad→qd_municipio, qd_celular→qd_telefono, qd_numeroCaso→qd_idCasoBPM, qd_rol→qd_rolRadicador, etc.) SCR-002	qd_canalRecepcion→qd_canal, qd_asunto→qd_motivoSFC, qd_descripcionQueja→qd_textoQueja, granulares en vez de qd_nombreConsumidor SCR-003 / SCR-004	prefijos ef_/et_ → qd_+técnico SCR-0051 / SCR-0052	granulares (nombre, identificación, instancia), qd_resumen→qd_motivoSFC; SCR-0052 además qd_areaAsignada→qd_areaResponsable, qd_responsableAsignado→qd_usuarioResponsable SCR-008	qd_idCasoSFC→qd_codigoSFC SCR-010	prefijo qd_ agregado a las 17 variables + qd_validacionNomenclatura SCR-009 / SCR-011 / SCR-012	sin cambios (ya correctas)
</commit_message>
<xml_diff>
--- a/pm4-app/insumos/Anexo02_Mockups_TOBE_QuejaDirectas_v3_0.xlsx
+++ b/pm4-app/insumos/Anexo02_Mockups_TOBE_QuejaDirectas_v3_0.xlsx
@@ -10041,7 +10041,7 @@
       </c>
       <c r="D73" s="80" t="inlineStr">
         <is>
-          <t>textoQueja &lt; 50 o &gt; 2000 caracteres</t>
+          <t>qd_textoQueja &lt; 50 o &gt; 2000 caracteres</t>
         </is>
       </c>
       <c r="F73" s="80" t="inlineStr">
@@ -10272,7 +10272,7 @@
       </c>
       <c r="D80" s="80" t="inlineStr">
         <is>
-          <t>numeroIdentificacion no cumple formato por tipo doc</t>
+          <t>qd_numeroIdentificacion no cumple formato por tipo doc</t>
         </is>
       </c>
       <c r="F80" s="80" t="inlineStr">
@@ -11656,7 +11656,7 @@
       </c>
       <c r="D48" s="80" t="inlineStr">
         <is>
-          <t>numeroIdentificacion contiene letras o longitud &lt;6 o &gt;15</t>
+          <t>qd_numeroIdentificacion contiene letras o longitud &lt;6 o &gt;15</t>
         </is>
       </c>
       <c r="F48" s="80" t="inlineStr">
@@ -11722,7 +11722,7 @@
       </c>
       <c r="D50" s="80" t="inlineStr">
         <is>
-          <t>resumen o nombreConsumidor contienen caracteres no permitidos SFC</t>
+          <t>qd_nombres, qd_apellidos o qd_razonSocial contienen caracteres no permitidos SFC</t>
         </is>
       </c>
       <c r="F50" s="80" t="inlineStr">
@@ -15611,7 +15611,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="20.1" customHeight="1" s="105">
-      <c r="B1" s="147" t="inlineStr">
+      <c r="B1" s="154" t="inlineStr">
         <is>
           <t>SCR-0051 — Flujo Combinado — Detalle / Reasignación / Respuesta</t>
         </is>
@@ -15625,7 +15625,7 @@
       <c r="I1" s="111" t="n"/>
     </row>
     <row r="2" ht="14.1" customHeight="1" s="105">
-      <c r="B2" s="148" t="inlineStr">
+      <c r="B2" s="155" t="inlineStr">
         <is>
           <t>Proceso: Gestión de Quejas Directas | ACZ-QD-001  |  Versión: 2.0 TO-BE | Mayo 2026</t>
         </is>
@@ -15639,7 +15639,7 @@
       <c r="I2" s="111" t="n"/>
     </row>
     <row r="3" ht="14.1" customHeight="1" s="105">
-      <c r="B3" s="148" t="inlineStr">
+      <c r="B3" s="155" t="inlineStr">
         <is>
           <t>Servicio: Atención al Consumidor Financiero – Zurich Seguros Colombia  |  Plataforma: ProcessMaker 4 BPMS</t>
         </is>
@@ -15654,7 +15654,7 @@
     </row>
     <row r="4" ht="5.1" customHeight="1" s="105"/>
     <row r="5" ht="14.1" customHeight="1" s="105">
-      <c r="B5" s="149" t="inlineStr">
+      <c r="B5" s="156" t="inlineStr">
         <is>
           <t>Proceso: SP2 — Gestionar Respuesta Interna y Revisión SAC  |  Tarea: SP2-T01 / T02 / T03 / T05  |  Rol: Analista SAC / Área Responsable  |  Estado: Radicado ante SFC / En análisis</t>
         </is>
@@ -15668,7 +15668,7 @@
       <c r="I5" s="111" t="n"/>
     </row>
     <row r="6" ht="14.1" customHeight="1" s="105">
-      <c r="B6" s="150" t="inlineStr">
+      <c r="B6" s="157" t="inlineStr">
         <is>
           <t>📖 HISTORIA DE USUARIO</t>
         </is>
@@ -15736,7 +15736,7 @@
       <c r="I9" s="111" t="n"/>
     </row>
     <row r="10" ht="14.1" customHeight="1" s="105">
-      <c r="B10" s="151" t="inlineStr">
+      <c r="B10" s="158" t="inlineStr">
         <is>
           <t>✅ CRITERIO DE ACEPTACIÓN</t>
         </is>
@@ -15805,7 +15805,7 @@
     </row>
     <row r="14" ht="5.1" customHeight="1" s="105"/>
     <row r="15" ht="14.1" customHeight="1" s="105">
-      <c r="B15" s="152" t="inlineStr">
+      <c r="B15" s="159" t="inlineStr">
         <is>
           <t>📋 CAMPOS DE LA PANTALLA</t>
         </is>
@@ -16988,7 +16988,7 @@
     </row>
     <row r="46" ht="5.1" customHeight="1" s="105"/>
     <row r="47" ht="14.1" customHeight="1" s="105">
-      <c r="B47" s="152" t="inlineStr">
+      <c r="B47" s="159" t="inlineStr">
         <is>
           <t>🎯 ACCIONES</t>
         </is>
@@ -17273,7 +17273,7 @@
     </row>
     <row r="57" ht="5.1" customHeight="1" s="105"/>
     <row r="58" ht="14.1" customHeight="1" s="105">
-      <c r="B58" s="153" t="inlineStr">
+      <c r="B58" s="163" t="inlineStr">
         <is>
           <t>⚠ REGLAS CRÍTICAS</t>
         </is>
@@ -17642,7 +17642,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="20.1" customHeight="1" s="105">
-      <c r="B1" s="147" t="inlineStr">
+      <c r="B1" s="154" t="inlineStr">
         <is>
           <t>SCR-0052 — Respuesta del Área Responsable</t>
         </is>
@@ -17656,7 +17656,7 @@
       <c r="I1" s="111" t="n"/>
     </row>
     <row r="2" ht="14.1" customHeight="1" s="105">
-      <c r="B2" s="148" t="inlineStr">
+      <c r="B2" s="155" t="inlineStr">
         <is>
           <t>Proceso: Gestión de Quejas Directas | ACZ-QD-001  |  Versión: 2.0 TO-BE | Mayo 2026</t>
         </is>
@@ -17670,7 +17670,7 @@
       <c r="I2" s="111" t="n"/>
     </row>
     <row r="3" ht="14.1" customHeight="1" s="105">
-      <c r="B3" s="148" t="inlineStr">
+      <c r="B3" s="155" t="inlineStr">
         <is>
           <t>Servicio: Atención al Consumidor Financiero – Zurich Seguros Colombia  |  Plataforma: ProcessMaker 4 BPMS</t>
         </is>
@@ -17685,7 +17685,7 @@
     </row>
     <row r="4" ht="5.1" customHeight="1" s="105"/>
     <row r="5" ht="14.1" customHeight="1" s="105">
-      <c r="B5" s="149" t="inlineStr">
+      <c r="B5" s="156" t="inlineStr">
         <is>
           <t>Proceso: SP2 — Gestionar Respuesta Interna y Revisión SAC  |  Tarea: SP2-T02  |  Rol: Área Responsable  |  Estado: En análisis</t>
         </is>
@@ -17699,7 +17699,7 @@
       <c r="I5" s="111" t="n"/>
     </row>
     <row r="6" ht="14.1" customHeight="1" s="105">
-      <c r="B6" s="150" t="inlineStr">
+      <c r="B6" s="157" t="inlineStr">
         <is>
           <t>📖 HISTORIA DE USUARIO</t>
         </is>
@@ -17767,7 +17767,7 @@
       <c r="I9" s="111" t="n"/>
     </row>
     <row r="10" ht="14.1" customHeight="1" s="105">
-      <c r="B10" s="151" t="inlineStr">
+      <c r="B10" s="158" t="inlineStr">
         <is>
           <t>✅ CRITERIO DE ACEPTACIÓN</t>
         </is>
@@ -17836,7 +17836,7 @@
     </row>
     <row r="14" ht="5.1" customHeight="1" s="105"/>
     <row r="15" ht="14.1" customHeight="1" s="105">
-      <c r="B15" s="152" t="inlineStr">
+      <c r="B15" s="159" t="inlineStr">
         <is>
           <t>📋 CAMPOS DE LA PANTALLA</t>
         </is>
@@ -18539,7 +18539,7 @@
     </row>
     <row r="34" ht="5.1" customHeight="1" s="105"/>
     <row r="35" ht="14.1" customHeight="1" s="105">
-      <c r="B35" s="152" t="inlineStr">
+      <c r="B35" s="159" t="inlineStr">
         <is>
           <t>🎯 ACCIONES</t>
         </is>
@@ -18674,7 +18674,7 @@
     </row>
     <row r="40" ht="5.1" customHeight="1" s="105"/>
     <row r="41" ht="14.1" customHeight="1" s="105">
-      <c r="B41" s="153" t="inlineStr">
+      <c r="B41" s="163" t="inlineStr">
         <is>
           <t>⚠ REGLAS CRÍTICAS</t>
         </is>
@@ -29519,7 +29519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q254"/>
+  <dimension ref="B1:Q254"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="14.45"/>
   <cols>
     <col width="3" customWidth="1" style="105" min="1" max="1"/>
@@ -29672,7 +29672,7 @@
       </c>
       <c r="G6" s="20" t="inlineStr">
         <is>
-          <t>idCasoBPM</t>
+          <t>qd_idCasoBPM</t>
         </is>
       </c>
       <c r="H6" s="20" t="inlineStr">
@@ -29750,7 +29750,7 @@
       </c>
       <c r="G7" s="20" t="inlineStr">
         <is>
-          <t>canalRecepcion</t>
+          <t>qd_canal</t>
         </is>
       </c>
       <c r="H7" s="20" t="inlineStr">
@@ -29832,7 +29832,7 @@
       </c>
       <c r="G8" s="20" t="inlineStr">
         <is>
-          <t>fechaCreacion</t>
+          <t>qd_fechaCreacion</t>
         </is>
       </c>
       <c r="H8" s="20" t="inlineStr">
@@ -29910,7 +29910,7 @@
       </c>
       <c r="G9" s="20" t="inlineStr">
         <is>
-          <t>nombreConsumidor</t>
+          <t>qd_nombres + qd_apellidos / qd_razonSocial</t>
         </is>
       </c>
       <c r="H9" s="20" t="inlineStr">
@@ -29984,7 +29984,7 @@
       </c>
       <c r="G10" s="20" t="inlineStr">
         <is>
-          <t>tipoIdentificacion</t>
+          <t>qd_tipoIdentificacion</t>
         </is>
       </c>
       <c r="H10" s="20" t="inlineStr">
@@ -30066,7 +30066,7 @@
       </c>
       <c r="G11" s="20" t="inlineStr">
         <is>
-          <t>numeroIdentificacion</t>
+          <t>qd_numeroIdentificacion</t>
         </is>
       </c>
       <c r="H11" s="20" t="inlineStr">
@@ -30140,7 +30140,7 @@
       </c>
       <c r="G12" s="20" t="inlineStr">
         <is>
-          <t>correoElectronico</t>
+          <t>qd_correoElectronico</t>
         </is>
       </c>
       <c r="H12" s="20" t="inlineStr">
@@ -30218,7 +30218,7 @@
       </c>
       <c r="G13" s="20" t="inlineStr">
         <is>
-          <t>tipoPersona</t>
+          <t>qd_tipoPersona</t>
         </is>
       </c>
       <c r="H13" s="20" t="inlineStr">
@@ -30300,7 +30300,7 @@
       </c>
       <c r="G14" s="20" t="inlineStr">
         <is>
-          <t>codigoPais</t>
+          <t>qd_codigoPais</t>
         </is>
       </c>
       <c r="H14" s="20" t="inlineStr">
@@ -30382,7 +30382,7 @@
       </c>
       <c r="G15" s="20" t="inlineStr">
         <is>
-          <t>departamento</t>
+          <t>qd_departamento</t>
         </is>
       </c>
       <c r="H15" s="20" t="inlineStr">
@@ -30464,7 +30464,7 @@
       </c>
       <c r="G16" s="20" t="inlineStr">
         <is>
-          <t>municipio</t>
+          <t>qd_municipio</t>
         </is>
       </c>
       <c r="H16" s="20" t="inlineStr">
@@ -30546,7 +30546,7 @@
       </c>
       <c r="G17" s="20" t="inlineStr">
         <is>
-          <t>resumen</t>
+          <t>qd_motivoSFC</t>
         </is>
       </c>
       <c r="H17" s="20" t="inlineStr">
@@ -30620,7 +30620,7 @@
       </c>
       <c r="G18" s="20" t="inlineStr">
         <is>
-          <t>textoQueja</t>
+          <t>qd_textoQueja</t>
         </is>
       </c>
       <c r="H18" s="20" t="inlineStr">
@@ -30694,7 +30694,7 @@
       </c>
       <c r="G19" s="20" t="inlineStr">
         <is>
-          <t>productoSFC</t>
+          <t>qd_productoSFC</t>
         </is>
       </c>
       <c r="H19" s="20" t="inlineStr">
@@ -30776,7 +30776,7 @@
       </c>
       <c r="G20" s="20" t="inlineStr">
         <is>
-          <t>motivoSFC</t>
+          <t>qd_motivoSFC</t>
         </is>
       </c>
       <c r="H20" s="20" t="inlineStr">
@@ -30858,7 +30858,7 @@
       </c>
       <c r="G21" s="20" t="inlineStr">
         <is>
-          <t>tipoSolicitudInterno</t>
+          <t>qd_tipoSolicitudInterno</t>
         </is>
       </c>
       <c r="H21" s="20" t="inlineStr">
@@ -30940,7 +30940,7 @@
       </c>
       <c r="G22" s="20" t="inlineStr">
         <is>
-          <t>instanciaRecepcion</t>
+          <t>qd_instanciaRecepcion</t>
         </is>
       </c>
       <c r="H22" s="20" t="inlineStr">
@@ -31018,7 +31018,7 @@
       </c>
       <c r="G23" s="20" t="inlineStr">
         <is>
-          <t>puntoRecepcion</t>
+          <t>qd_puntoRecepcion</t>
         </is>
       </c>
       <c r="H23" s="20" t="inlineStr">
@@ -31096,7 +31096,7 @@
       </c>
       <c r="G24" s="20" t="inlineStr">
         <is>
-          <t>admision</t>
+          <t>qd_admision</t>
         </is>
       </c>
       <c r="H24" s="20" t="inlineStr">
@@ -31174,7 +31174,7 @@
       </c>
       <c r="G25" s="20" t="inlineStr">
         <is>
-          <t>enteControl</t>
+          <t>qd_enteControl</t>
         </is>
       </c>
       <c r="H25" s="20" t="inlineStr">
@@ -31252,7 +31252,7 @@
       </c>
       <c r="G26" s="20" t="inlineStr">
         <is>
-          <t>incluyeAnexos</t>
+          <t>qd_incluyeAnexos</t>
         </is>
       </c>
       <c r="H26" s="20" t="inlineStr">
@@ -31330,7 +31330,7 @@
       </c>
       <c r="G27" s="20" t="inlineStr">
         <is>
-          <t>adjuntosQueja</t>
+          <t>qd_adjuntosQueja</t>
         </is>
       </c>
       <c r="H27" s="20" t="inlineStr">
@@ -31404,7 +31404,7 @@
       </c>
       <c r="G28" s="20" t="inlineStr">
         <is>
-          <t>idCasoBPM</t>
+          <t>qd_idCasoBPM</t>
         </is>
       </c>
       <c r="H28" s="20" t="inlineStr">
@@ -31478,7 +31478,7 @@
       </c>
       <c r="G29" s="20" t="inlineStr">
         <is>
-          <t>canalRecepcion</t>
+          <t>qd_canal</t>
         </is>
       </c>
       <c r="H29" s="20" t="inlineStr">
@@ -31552,7 +31552,7 @@
       </c>
       <c r="G30" s="20" t="inlineStr">
         <is>
-          <t>slaRestante</t>
+          <t>qd_slaRestante</t>
         </is>
       </c>
       <c r="H30" s="20" t="inlineStr">
@@ -31630,7 +31630,7 @@
       </c>
       <c r="G31" s="20" t="inlineStr">
         <is>
-          <t>contadorErrores</t>
+          <t>qd_contadorErrores</t>
         </is>
       </c>
       <c r="H31" s="20" t="inlineStr">
@@ -31708,7 +31708,7 @@
       </c>
       <c r="G32" s="20" t="inlineStr">
         <is>
-          <t>panelErrores</t>
+          <t>qd_panelErrores</t>
         </is>
       </c>
       <c r="H32" s="20" t="inlineStr">
@@ -31786,7 +31786,7 @@
       </c>
       <c r="G33" s="20" t="inlineStr">
         <is>
-          <t>camposConError</t>
+          <t>qd_camposConError</t>
         </is>
       </c>
       <c r="H33" s="20" t="inlineStr">
@@ -31864,7 +31864,7 @@
       </c>
       <c r="G34" s="20" t="inlineStr">
         <is>
-          <t>codigoErrorSFC</t>
+          <t>qd_codigoErrorSFC</t>
         </is>
       </c>
       <c r="H34" s="20" t="inlineStr">
@@ -31942,7 +31942,7 @@
       </c>
       <c r="G35" s="20" t="inlineStr">
         <is>
-          <t>campoAfectado</t>
+          <t>qd_campoAfectado</t>
         </is>
       </c>
       <c r="H35" s="20" t="inlineStr">
@@ -32020,7 +32020,7 @@
       </c>
       <c r="G36" s="20" t="inlineStr">
         <is>
-          <t>valorRechazado</t>
+          <t>qd_valorRechazado</t>
         </is>
       </c>
       <c r="H36" s="20" t="inlineStr">
@@ -32098,7 +32098,7 @@
       </c>
       <c r="G37" s="20" t="inlineStr">
         <is>
-          <t>mensajeErrorSFC</t>
+          <t>qd_mensajeErrorSFC</t>
         </is>
       </c>
       <c r="H37" s="20" t="inlineStr">
@@ -32176,7 +32176,7 @@
       </c>
       <c r="G38" s="20" t="inlineStr">
         <is>
-          <t>numerIntentoM1M2</t>
+          <t>qd_numeroIntentoM1M2</t>
         </is>
       </c>
       <c r="H38" s="20" t="inlineStr">
@@ -32250,7 +32250,7 @@
       </c>
       <c r="G39" s="20" t="inlineStr">
         <is>
-          <t>fechaRechazo</t>
+          <t>qd_fechaRechazo</t>
         </is>
       </c>
       <c r="H39" s="20" t="inlineStr">
@@ -32328,7 +32328,7 @@
       </c>
       <c r="G40" s="20" t="inlineStr">
         <is>
-          <t>campoCorreccion</t>
+          <t>qd_campoCorreccion</t>
         </is>
       </c>
       <c r="H40" s="20" t="inlineStr">
@@ -32406,7 +32406,7 @@
       </c>
       <c r="G41" s="20" t="inlineStr">
         <is>
-          <t>justificacionCorreccion</t>
+          <t>qd_justificacionCorreccion</t>
         </is>
       </c>
       <c r="H41" s="20" t="inlineStr">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="G42" s="20" t="inlineStr">
         <is>
-          <t>historialIntentos</t>
+          <t>qd_historialIntentos</t>
         </is>
       </c>
       <c r="H42" s="20" t="inlineStr">
@@ -32562,7 +32562,7 @@
       </c>
       <c r="G43" s="20" t="inlineStr">
         <is>
-          <t>codigoHTTP</t>
+          <t>qd_codigoHTTP</t>
         </is>
       </c>
       <c r="H43" s="20" t="inlineStr">
@@ -32640,7 +32640,7 @@
       </c>
       <c r="G44" s="20" t="inlineStr">
         <is>
-          <t>tipoError</t>
+          <t>qd_tipoError</t>
         </is>
       </c>
       <c r="H44" s="20" t="inlineStr">
@@ -32718,7 +32718,7 @@
       </c>
       <c r="G45" s="20" t="inlineStr">
         <is>
-          <t>mensajeTecnicoAPI</t>
+          <t>qd_mensajeTecnicoAPI</t>
         </is>
       </c>
       <c r="H45" s="20" t="inlineStr">
@@ -32796,7 +32796,7 @@
       </c>
       <c r="G46" s="20" t="inlineStr">
         <is>
-          <t>endpointInvocado</t>
+          <t>qd_endpointInvocado</t>
         </is>
       </c>
       <c r="H46" s="20" t="inlineStr">
@@ -32874,7 +32874,7 @@
       </c>
       <c r="G47" s="20" t="inlineStr">
         <is>
-          <t>payloadEnviado</t>
+          <t>qd_payloadEnviado</t>
         </is>
       </c>
       <c r="H47" s="20" t="inlineStr">
@@ -32952,7 +32952,7 @@
       </c>
       <c r="G48" s="20" t="inlineStr">
         <is>
-          <t>numeroIntento</t>
+          <t>qd_numeroIntento</t>
         </is>
       </c>
       <c r="H48" s="20" t="inlineStr">
@@ -33026,7 +33026,7 @@
       </c>
       <c r="G49" s="20" t="inlineStr">
         <is>
-          <t>causaRaiz</t>
+          <t>qd_causaRaiz</t>
         </is>
       </c>
       <c r="H49" s="20" t="inlineStr">
@@ -33104,7 +33104,7 @@
       </c>
       <c r="G50" s="20" t="inlineStr">
         <is>
-          <t>correccionAplicada</t>
+          <t>qd_correccionAplicada</t>
         </is>
       </c>
       <c r="H50" s="20" t="inlineStr">
@@ -33182,7 +33182,7 @@
       </c>
       <c r="G51" s="20" t="inlineStr">
         <is>
-          <t>requiereAjustePayload</t>
+          <t>qd_requiereAjustePayload</t>
         </is>
       </c>
       <c r="H51" s="20" t="inlineStr">
@@ -33256,7 +33256,7 @@
       </c>
       <c r="G52" s="20" t="inlineStr">
         <is>
-          <t>idCasoBPM</t>
+          <t>qd_idCasoBPM</t>
         </is>
       </c>
       <c r="H52" s="20" t="inlineStr">
@@ -33330,7 +33330,7 @@
       </c>
       <c r="G53" s="20" t="inlineStr">
         <is>
-          <t>codigoSFC</t>
+          <t>qd_codigoSFC</t>
         </is>
       </c>
       <c r="H53" s="20" t="inlineStr">
@@ -33408,7 +33408,7 @@
       </c>
       <c r="G54" s="20" t="inlineStr">
         <is>
-          <t>estadoCaso</t>
+          <t>qd_estadoCaso</t>
         </is>
       </c>
       <c r="H54" s="20" t="inlineStr">
@@ -33482,7 +33482,7 @@
       </c>
       <c r="G55" s="20" t="inlineStr">
         <is>
-          <t>slaRestante</t>
+          <t>qd_slaRestante</t>
         </is>
       </c>
       <c r="H55" s="20" t="inlineStr">
@@ -33560,7 +33560,7 @@
       </c>
       <c r="G56" s="20" t="inlineStr">
         <is>
-          <t>fechaLimite</t>
+          <t>qd_fechaLimite</t>
         </is>
       </c>
       <c r="H56" s="20" t="inlineStr">
@@ -33638,7 +33638,7 @@
       </c>
       <c r="G57" s="20" t="inlineStr">
         <is>
-          <t>responsableActual</t>
+          <t>qd_responsableActual</t>
         </is>
       </c>
       <c r="H57" s="20" t="inlineStr">
@@ -33712,7 +33712,7 @@
       </c>
       <c r="G58" s="20" t="inlineStr">
         <is>
-          <t>nombreConsumidor</t>
+          <t>qd_nombres + qd_apellidos / qd_razonSocial</t>
         </is>
       </c>
       <c r="H58" s="20" t="inlineStr">
@@ -33786,7 +33786,7 @@
       </c>
       <c r="G59" s="20" t="inlineStr">
         <is>
-          <t>identificacion</t>
+          <t>qd_tipoIdentificacion + qd_numeroIdentificacion</t>
         </is>
       </c>
       <c r="H59" s="20" t="inlineStr">
@@ -33860,7 +33860,7 @@
       </c>
       <c r="G60" s="20" t="inlineStr">
         <is>
-          <t>correoElectronico</t>
+          <t>qd_correoElectronico</t>
         </is>
       </c>
       <c r="H60" s="20" t="inlineStr">
@@ -33934,7 +33934,7 @@
       </c>
       <c r="G61" s="20" t="inlineStr">
         <is>
-          <t>tipoPersona</t>
+          <t>qd_tipoPersona</t>
         </is>
       </c>
       <c r="H61" s="20" t="inlineStr">
@@ -34008,7 +34008,7 @@
       </c>
       <c r="G62" s="20" t="inlineStr">
         <is>
-          <t>canal</t>
+          <t>qd_canal</t>
         </is>
       </c>
       <c r="H62" s="20" t="inlineStr">
@@ -34082,7 +34082,7 @@
       </c>
       <c r="G63" s="20" t="inlineStr">
         <is>
-          <t>productoSFC</t>
+          <t>qd_productoSFC</t>
         </is>
       </c>
       <c r="H63" s="20" t="inlineStr">
@@ -34156,7 +34156,7 @@
       </c>
       <c r="G64" s="20" t="inlineStr">
         <is>
-          <t>motivoSFC</t>
+          <t>qd_motivoSFC</t>
         </is>
       </c>
       <c r="H64" s="20" t="inlineStr">
@@ -34230,7 +34230,7 @@
       </c>
       <c r="G65" s="20" t="inlineStr">
         <is>
-          <t>instanciaPunto</t>
+          <t>qd_instanciaRecepcion</t>
         </is>
       </c>
       <c r="H65" s="20" t="inlineStr">
@@ -34304,7 +34304,7 @@
       </c>
       <c r="G66" s="20" t="inlineStr">
         <is>
-          <t>admision</t>
+          <t>qd_admision</t>
         </is>
       </c>
       <c r="H66" s="20" t="inlineStr">
@@ -34378,7 +34378,7 @@
       </c>
       <c r="G67" s="20" t="inlineStr">
         <is>
-          <t>enteControl</t>
+          <t>qd_enteControl</t>
         </is>
       </c>
       <c r="H67" s="20" t="inlineStr">
@@ -34452,7 +34452,7 @@
       </c>
       <c r="G68" s="20" t="inlineStr">
         <is>
-          <t>resumen</t>
+          <t>qd_motivoSFC</t>
         </is>
       </c>
       <c r="H68" s="20" t="inlineStr">
@@ -34526,7 +34526,7 @@
       </c>
       <c r="G69" s="20" t="inlineStr">
         <is>
-          <t>textoQueja</t>
+          <t>qd_textoQueja</t>
         </is>
       </c>
       <c r="H69" s="20" t="inlineStr">
@@ -34600,7 +34600,7 @@
       </c>
       <c r="G70" s="20" t="inlineStr">
         <is>
-          <t>adjuntosCliente</t>
+          <t>qd_adjuntosCliente</t>
         </is>
       </c>
       <c r="H70" s="20" t="inlineStr">
@@ -34678,7 +34678,7 @@
       </c>
       <c r="G71" s="20" t="inlineStr">
         <is>
-          <t>estadoSS</t>
+          <t>qd_estadoSS</t>
         </is>
       </c>
       <c r="H71" s="20" t="inlineStr">
@@ -34756,7 +34756,7 @@
       </c>
       <c r="G72" s="20" t="inlineStr">
         <is>
-          <t>intentosM1M2</t>
+          <t>qd_intentosM1M2</t>
         </is>
       </c>
       <c r="H72" s="20" t="inlineStr">
@@ -34830,7 +34830,7 @@
       </c>
       <c r="G73" s="20" t="inlineStr">
         <is>
-          <t>fechaRadicacion</t>
+          <t>qd_fechaRadicacion</t>
         </is>
       </c>
       <c r="H73" s="20" t="inlineStr">
@@ -34908,7 +34908,7 @@
       </c>
       <c r="G74" s="20" t="inlineStr">
         <is>
-          <t>areaResponsable</t>
+          <t>qd_areaResponsable</t>
         </is>
       </c>
       <c r="H74" s="20" t="inlineStr">
@@ -34990,7 +34990,7 @@
       </c>
       <c r="G75" s="20" t="inlineStr">
         <is>
-          <t>usuarioResponsable</t>
+          <t>qd_usuarioResponsable</t>
         </is>
       </c>
       <c r="H75" s="20" t="inlineStr">
@@ -35072,7 +35072,7 @@
       </c>
       <c r="G76" s="20" t="inlineStr">
         <is>
-          <t>observacionesAsignacion</t>
+          <t>qd_observacionesAsignacion</t>
         </is>
       </c>
       <c r="H76" s="20" t="inlineStr">
@@ -35146,7 +35146,7 @@
       </c>
       <c r="G77" s="20" t="inlineStr">
         <is>
-          <t>responsableActual</t>
+          <t>qd_responsableActual</t>
         </is>
       </c>
       <c r="H77" s="20" t="inlineStr">
@@ -35220,7 +35220,7 @@
       </c>
       <c r="G78" s="20" t="inlineStr">
         <is>
-          <t>areaDestino</t>
+          <t>qd_areaDestino</t>
         </is>
       </c>
       <c r="H78" s="20" t="inlineStr">
@@ -35298,7 +35298,7 @@
       </c>
       <c r="G79" s="20" t="inlineStr">
         <is>
-          <t>nuevoResponsable</t>
+          <t>qd_nuevoResponsable</t>
         </is>
       </c>
       <c r="H79" s="20" t="inlineStr">
@@ -35380,7 +35380,7 @@
       </c>
       <c r="G80" s="20" t="inlineStr">
         <is>
-          <t>motivoReasignacion</t>
+          <t>qd_motivoReasignacion</t>
         </is>
       </c>
       <c r="H80" s="20" t="inlineStr">
@@ -35458,7 +35458,7 @@
       </c>
       <c r="G81" s="20" t="inlineStr">
         <is>
-          <t>observacionesReasignacion</t>
+          <t>qd_observacionesReasignacion</t>
         </is>
       </c>
       <c r="H81" s="20" t="inlineStr">
@@ -35536,7 +35536,7 @@
       </c>
       <c r="G82" s="20" t="inlineStr">
         <is>
-          <t>historialAsignaciones</t>
+          <t>qd_historialAsignaciones</t>
         </is>
       </c>
       <c r="H82" s="20" t="inlineStr">
@@ -35614,7 +35614,7 @@
       </c>
       <c r="G83" s="20" t="inlineStr">
         <is>
-          <t>idCasoSFC</t>
+          <t>qd_codigoSFC</t>
         </is>
       </c>
       <c r="H83" s="20" t="inlineStr">
@@ -35688,7 +35688,7 @@
       </c>
       <c r="G84" s="20" t="inlineStr">
         <is>
-          <t>slaRestante</t>
+          <t>qd_slaRestante</t>
         </is>
       </c>
       <c r="H84" s="20" t="inlineStr">
@@ -35766,7 +35766,7 @@
       </c>
       <c r="G85" s="20" t="inlineStr">
         <is>
-          <t>estadoCaso</t>
+          <t>qd_estadoCaso</t>
         </is>
       </c>
       <c r="H85" s="20" t="inlineStr">
@@ -35840,7 +35840,7 @@
       </c>
       <c r="G86" s="20" t="inlineStr">
         <is>
-          <t>productoMotivo</t>
+          <t>qd_productoMotivo</t>
         </is>
       </c>
       <c r="H86" s="20" t="inlineStr">
@@ -35914,7 +35914,7 @@
       </c>
       <c r="G87" s="20" t="inlineStr">
         <is>
-          <t>nombreConsumidor</t>
+          <t>qd_nombres + qd_apellidos / qd_razonSocial</t>
         </is>
       </c>
       <c r="H87" s="20" t="inlineStr">
@@ -35988,7 +35988,7 @@
       </c>
       <c r="G88" s="20" t="inlineStr">
         <is>
-          <t>textoQueja</t>
+          <t>qd_textoQueja</t>
         </is>
       </c>
       <c r="H88" s="20" t="inlineStr">
@@ -36062,7 +36062,7 @@
       </c>
       <c r="G89" s="20" t="inlineStr">
         <is>
-          <t>observacionesSAC</t>
+          <t>qd_observacionesSAC</t>
         </is>
       </c>
       <c r="H89" s="20" t="inlineStr">
@@ -36140,7 +36140,7 @@
       </c>
       <c r="G90" s="20" t="inlineStr">
         <is>
-          <t>versionRevision</t>
+          <t>qd_versionRevision</t>
         </is>
       </c>
       <c r="H90" s="20" t="inlineStr">
@@ -36218,7 +36218,7 @@
       </c>
       <c r="G91" s="20" t="inlineStr">
         <is>
-          <t>causaRaiz</t>
+          <t>qd_causaRaiz</t>
         </is>
       </c>
       <c r="H91" s="20" t="inlineStr">
@@ -36292,7 +36292,7 @@
       </c>
       <c r="G92" s="20" t="inlineStr">
         <is>
-          <t>posicionZurich</t>
+          <t>qd_posicionZurich</t>
         </is>
       </c>
       <c r="H92" s="20" t="inlineStr">
@@ -36366,7 +36366,7 @@
       </c>
       <c r="G93" s="20" t="inlineStr">
         <is>
-          <t>respuestaCliente</t>
+          <t>qd_respuestaCliente</t>
         </is>
       </c>
       <c r="H93" s="20" t="inlineStr">
@@ -36444,7 +36444,7 @@
       </c>
       <c r="G94" s="20" t="inlineStr">
         <is>
-          <t>accionesTomadas</t>
+          <t>qd_accionesTomadas</t>
         </is>
       </c>
       <c r="H94" s="20" t="inlineStr">
@@ -36518,7 +36518,7 @@
       </c>
       <c r="G95" s="20" t="inlineStr">
         <is>
-          <t>reconocimiento</t>
+          <t>qd_reconocimiento</t>
         </is>
       </c>
       <c r="H95" s="20" t="inlineStr">
@@ -36592,7 +36592,7 @@
       </c>
       <c r="G96" s="20" t="inlineStr">
         <is>
-          <t>adjuntosSoporte</t>
+          <t>qd_adjuntosSoporte</t>
         </is>
       </c>
       <c r="H96" s="20" t="inlineStr">
@@ -36670,7 +36670,7 @@
       </c>
       <c r="G97" s="20" t="inlineStr">
         <is>
-          <t>idCasoSFC</t>
+          <t>qd_codigoSFC</t>
         </is>
       </c>
       <c r="H97" s="20" t="inlineStr">
@@ -36744,7 +36744,7 @@
       </c>
       <c r="G98" s="20" t="inlineStr">
         <is>
-          <t>slaRestante</t>
+          <t>qd_slaRestante</t>
         </is>
       </c>
       <c r="H98" s="20" t="inlineStr">
@@ -36818,7 +36818,7 @@
       </c>
       <c r="G99" s="20" t="inlineStr">
         <is>
-          <t>versionRevision</t>
+          <t>qd_versionRevision</t>
         </is>
       </c>
       <c r="H99" s="20" t="inlineStr">
@@ -36892,7 +36892,7 @@
       </c>
       <c r="G100" s="20" t="inlineStr">
         <is>
-          <t>areaResponsable</t>
+          <t>qd_areaResponsable</t>
         </is>
       </c>
       <c r="H100" s="20" t="inlineStr">
@@ -36966,7 +36966,7 @@
       </c>
       <c r="G101" s="20" t="inlineStr">
         <is>
-          <t>fechaElaboracion</t>
+          <t>qd_fechaElaboracion</t>
         </is>
       </c>
       <c r="H101" s="20" t="inlineStr">
@@ -37040,7 +37040,7 @@
       </c>
       <c r="G102" s="20" t="inlineStr">
         <is>
-          <t>respuestaCliente</t>
+          <t>qd_respuestaCliente</t>
         </is>
       </c>
       <c r="H102" s="20" t="inlineStr">
@@ -37114,7 +37114,7 @@
       </c>
       <c r="G103" s="20" t="inlineStr">
         <is>
-          <t>accionesTomadas</t>
+          <t>qd_accionesTomadas</t>
         </is>
       </c>
       <c r="H103" s="20" t="inlineStr">
@@ -37188,7 +37188,7 @@
       </c>
       <c r="G104" s="20" t="inlineStr">
         <is>
-          <t>reconocimiento</t>
+          <t>qd_reconocimiento</t>
         </is>
       </c>
       <c r="H104" s="20" t="inlineStr">
@@ -37262,7 +37262,7 @@
       </c>
       <c r="G105" s="20" t="inlineStr">
         <is>
-          <t>adjuntosSoporte</t>
+          <t>qd_adjuntosSoporte</t>
         </is>
       </c>
       <c r="H105" s="20" t="inlineStr">
@@ -37340,7 +37340,7 @@
       </c>
       <c r="G106" s="20" t="inlineStr">
         <is>
-          <t>observacionesSAC</t>
+          <t>qd_observacionesSAC</t>
         </is>
       </c>
       <c r="H106" s="20" t="inlineStr">
@@ -37418,7 +37418,7 @@
       </c>
       <c r="G107" s="20" t="inlineStr">
         <is>
-          <t>codigoSFC</t>
+          <t>qd_codigoSFC</t>
         </is>
       </c>
       <c r="H107" s="20" t="inlineStr">
@@ -37492,7 +37492,7 @@
       </c>
       <c r="G108" s="20" t="inlineStr">
         <is>
-          <t>canal</t>
+          <t>qd_canal</t>
         </is>
       </c>
       <c r="H108" s="20" t="inlineStr">
@@ -37570,7 +37570,7 @@
       </c>
       <c r="G109" s="20" t="inlineStr">
         <is>
-          <t>productoSFC</t>
+          <t>qd_productoSFC</t>
         </is>
       </c>
       <c r="H109" s="20" t="inlineStr">
@@ -37648,7 +37648,7 @@
       </c>
       <c r="G110" s="20" t="inlineStr">
         <is>
-          <t>motivoSFC</t>
+          <t>qd_motivoSFC</t>
         </is>
       </c>
       <c r="H110" s="20" t="inlineStr">
@@ -37726,7 +37726,7 @@
       </c>
       <c r="G111" s="20" t="inlineStr">
         <is>
-          <t>admision</t>
+          <t>qd_admision</t>
         </is>
       </c>
       <c r="H111" s="20" t="inlineStr">
@@ -37804,7 +37804,7 @@
       </c>
       <c r="G112" s="20" t="inlineStr">
         <is>
-          <t>enteControl</t>
+          <t>qd_enteControl</t>
         </is>
       </c>
       <c r="H112" s="20" t="inlineStr">
@@ -37882,7 +37882,7 @@
       </c>
       <c r="G113" s="20" t="inlineStr">
         <is>
-          <t>sexo</t>
+          <t>qd_sexo</t>
         </is>
       </c>
       <c r="H113" s="20" t="inlineStr">
@@ -37960,7 +37960,7 @@
       </c>
       <c r="G114" s="20" t="inlineStr">
         <is>
-          <t>lgbtiq</t>
+          <t>qd_lgbtiq</t>
         </is>
       </c>
       <c r="H114" s="20" t="inlineStr">
@@ -38042,7 +38042,7 @@
       </c>
       <c r="G115" s="20" t="inlineStr">
         <is>
-          <t>condicionEspecial</t>
+          <t>qd_condicionEspecial</t>
         </is>
       </c>
       <c r="H115" s="20" t="inlineStr">
@@ -38120,7 +38120,7 @@
       </c>
       <c r="G116" s="20" t="inlineStr">
         <is>
-          <t>productoDigital</t>
+          <t>qd_productoDigital</t>
         </is>
       </c>
       <c r="H116" s="20" t="inlineStr">
@@ -38198,7 +38198,7 @@
       </c>
       <c r="G117" s="20" t="inlineStr">
         <is>
-          <t>estadoQueja</t>
+          <t>qd_estadoQueja</t>
         </is>
       </c>
       <c r="H117" s="20" t="inlineStr">
@@ -38276,7 +38276,7 @@
       </c>
       <c r="G118" s="20" t="inlineStr">
         <is>
-          <t>favorabilidad</t>
+          <t>qd_favorabilidad</t>
         </is>
       </c>
       <c r="H118" s="20" t="inlineStr">
@@ -38358,7 +38358,7 @@
       </c>
       <c r="G119" s="20" t="inlineStr">
         <is>
-          <t>aceptacion</t>
+          <t>qd_aceptacion</t>
         </is>
       </c>
       <c r="H119" s="20" t="inlineStr">
@@ -38436,7 +38436,7 @@
       </c>
       <c r="G120" s="20" t="inlineStr">
         <is>
-          <t>rectificacion</t>
+          <t>qd_rectificacion</t>
         </is>
       </c>
       <c r="H120" s="20" t="inlineStr">
@@ -38514,7 +38514,7 @@
       </c>
       <c r="G121" s="20" t="inlineStr">
         <is>
-          <t>desistimiento</t>
+          <t>qd_desistimiento</t>
         </is>
       </c>
       <c r="H121" s="20" t="inlineStr">
@@ -38592,7 +38592,7 @@
       </c>
       <c r="G122" s="20" t="inlineStr">
         <is>
-          <t>tutela</t>
+          <t>qd_tutela</t>
         </is>
       </c>
       <c r="H122" s="20" t="inlineStr">
@@ -38670,7 +38670,7 @@
       </c>
       <c r="G123" s="20" t="inlineStr">
         <is>
-          <t>marcacion</t>
+          <t>qd_marcacion</t>
         </is>
       </c>
       <c r="H123" s="20" t="inlineStr">
@@ -38748,7 +38748,7 @@
       </c>
       <c r="G124" s="20" t="inlineStr">
         <is>
-          <t>quejaExpres</t>
+          <t>qd_quejaExpres</t>
         </is>
       </c>
       <c r="H124" s="20" t="inlineStr">
@@ -38826,7 +38826,7 @@
       </c>
       <c r="G125" s="20" t="inlineStr">
         <is>
-          <t>relacionadaFraude</t>
+          <t>qd_relacionadaFraude</t>
         </is>
       </c>
       <c r="H125" s="20" t="inlineStr">
@@ -38904,7 +38904,7 @@
       </c>
       <c r="G126" s="20" t="inlineStr">
         <is>
-          <t>tipoFraude</t>
+          <t>qd_tipoFraude</t>
         </is>
       </c>
       <c r="H126" s="20" t="inlineStr">
@@ -38986,7 +38986,7 @@
       </c>
       <c r="G127" s="20" t="inlineStr">
         <is>
-          <t>modalidadFraude</t>
+          <t>qd_modalidadFraude</t>
         </is>
       </c>
       <c r="H127" s="20" t="inlineStr">
@@ -39068,7 +39068,7 @@
       </c>
       <c r="G128" s="20" t="inlineStr">
         <is>
-          <t>montoReclamado</t>
+          <t>qd_montoReclamado</t>
         </is>
       </c>
       <c r="H128" s="20" t="inlineStr">
@@ -39146,7 +39146,7 @@
       </c>
       <c r="G129" s="20" t="inlineStr">
         <is>
-          <t>montoReconocido</t>
+          <t>qd_montoReconocido</t>
         </is>
       </c>
       <c r="H129" s="20" t="inlineStr">
@@ -39224,7 +39224,7 @@
       </c>
       <c r="G130" s="20" t="inlineStr">
         <is>
-          <t>incluyeAnexosQueja</t>
+          <t>qd_incluyeAnexosQueja</t>
         </is>
       </c>
       <c r="H130" s="20" t="inlineStr">
@@ -39302,7 +39302,7 @@
       </c>
       <c r="G131" s="20" t="inlineStr">
         <is>
-          <t>incluyeAdjuntoRespuesta</t>
+          <t>qd_incluyeAdjuntoRespuesta</t>
         </is>
       </c>
       <c r="H131" s="20" t="inlineStr">
@@ -39380,7 +39380,7 @@
       </c>
       <c r="G132" s="20" t="inlineStr">
         <is>
-          <t>pdfRespuestaFinal</t>
+          <t>qd_pdfRespuestaFinal</t>
         </is>
       </c>
       <c r="H132" s="20" t="inlineStr">
@@ -39458,7 +39458,7 @@
       </c>
       <c r="G133" s="20" t="inlineStr">
         <is>
-          <t>diasProrroga</t>
+          <t>qd_diasProrroga</t>
         </is>
       </c>
       <c r="H133" s="20" t="inlineStr">
@@ -39536,7 +39536,7 @@
       </c>
       <c r="G134" s="20" t="inlineStr">
         <is>
-          <t>estadoCierreM3</t>
+          <t>qd_estadoCierreM3</t>
         </is>
       </c>
       <c r="H134" s="20" t="inlineStr">
@@ -39614,7 +39614,7 @@
       </c>
       <c r="G135" s="20" t="inlineStr">
         <is>
-          <t>intentosCierreM3</t>
+          <t>qd_intentosCierreM3</t>
         </is>
       </c>
       <c r="H135" s="20" t="inlineStr">
@@ -39688,7 +39688,7 @@
       </c>
       <c r="G136" s="20" t="inlineStr">
         <is>
-          <t>ultimoError</t>
+          <t>qd_ultimoError</t>
         </is>
       </c>
       <c r="H136" s="20" t="inlineStr">
@@ -39766,7 +39766,7 @@
       </c>
       <c r="G137" s="20" t="inlineStr">
         <is>
-          <t>codigoSFC</t>
+          <t>qd_codigoSFC</t>
         </is>
       </c>
       <c r="H137" s="20" t="inlineStr">
@@ -39840,7 +39840,7 @@
       </c>
       <c r="G138" s="20" t="inlineStr">
         <is>
-          <t>estadoQueja</t>
+          <t>qd_estadoQueja</t>
         </is>
       </c>
       <c r="H138" s="20" t="inlineStr">
@@ -39918,7 +39918,7 @@
       </c>
       <c r="G139" s="20" t="inlineStr">
         <is>
-          <t>fechaActualizacion</t>
+          <t>qd_fechaActualizacion</t>
         </is>
       </c>
       <c r="H139" s="20" t="inlineStr">
@@ -39996,7 +39996,7 @@
       </c>
       <c r="G140" s="20" t="inlineStr">
         <is>
-          <t>fechaCierre</t>
+          <t>qd_fechaCierre</t>
         </is>
       </c>
       <c r="H140" s="20" t="inlineStr">
@@ -40074,7 +40074,7 @@
       </c>
       <c r="G141" s="20" t="inlineStr">
         <is>
-          <t>favorabilidad</t>
+          <t>qd_favorabilidad</t>
         </is>
       </c>
       <c r="H141" s="20" t="inlineStr">
@@ -40156,7 +40156,7 @@
       </c>
       <c r="G142" s="20" t="inlineStr">
         <is>
-          <t>aceptacion</t>
+          <t>qd_aceptacion</t>
         </is>
       </c>
       <c r="H142" s="20" t="inlineStr">
@@ -40238,7 +40238,7 @@
       </c>
       <c r="G143" s="20" t="inlineStr">
         <is>
-          <t>marcacion</t>
+          <t>qd_marcacion</t>
         </is>
       </c>
       <c r="H143" s="20" t="inlineStr">
@@ -40316,7 +40316,7 @@
       </c>
       <c r="G144" s="20" t="inlineStr">
         <is>
-          <t>quejaExpres</t>
+          <t>qd_quejaExpres</t>
         </is>
       </c>
       <c r="H144" s="20" t="inlineStr">
@@ -40394,7 +40394,7 @@
       </c>
       <c r="G145" s="20" t="inlineStr">
         <is>
-          <t>pdfRespuestaFinal</t>
+          <t>qd_pdfRespuestaFinal</t>
         </is>
       </c>
       <c r="H145" s="20" t="inlineStr">
@@ -40472,7 +40472,7 @@
       </c>
       <c r="G146" s="20" t="inlineStr">
         <is>
-          <t>validacionNomenclatura</t>
+          <t>qd_validacionNomenclatura</t>
         </is>
       </c>
       <c r="H146" s="20" t="inlineStr">
@@ -40550,7 +40550,7 @@
       </c>
       <c r="G147" s="20" t="inlineStr">
         <is>
-          <t>adjuntoRespuestaFinal</t>
+          <t>qd_adjuntoRespuestaFinal</t>
         </is>
       </c>
       <c r="H147" s="20" t="inlineStr">
@@ -40624,7 +40624,7 @@
       </c>
       <c r="G148" s="20" t="inlineStr">
         <is>
-          <t>relacionadaFraude</t>
+          <t>qd_relacionadaFraude</t>
         </is>
       </c>
       <c r="H148" s="20" t="inlineStr">
@@ -40702,7 +40702,7 @@
       </c>
       <c r="G149" s="20" t="inlineStr">
         <is>
-          <t>tipoFraude</t>
+          <t>qd_tipoFraude</t>
         </is>
       </c>
       <c r="H149" s="20" t="inlineStr">
@@ -40776,7 +40776,7 @@
       </c>
       <c r="G150" s="20" t="inlineStr">
         <is>
-          <t>montoReclamado</t>
+          <t>qd_montoReclamado</t>
         </is>
       </c>
       <c r="H150" s="20" t="inlineStr">
@@ -40850,7 +40850,7 @@
       </c>
       <c r="G151" s="20" t="inlineStr">
         <is>
-          <t>montoReconocido</t>
+          <t>qd_montoReconocido</t>
         </is>
       </c>
       <c r="H151" s="20" t="inlineStr">
@@ -40924,7 +40924,7 @@
       </c>
       <c r="G152" s="20" t="inlineStr">
         <is>
-          <t>codigoHTTPProrroga</t>
+          <t>qd_codigoHTTPProrroga</t>
         </is>
       </c>
       <c r="H152" s="20" t="inlineStr">
@@ -40998,7 +40998,7 @@
       </c>
       <c r="G153" s="20" t="inlineStr">
         <is>
-          <t>tipoErrorProrroga</t>
+          <t>qd_tipoErrorProrroga</t>
         </is>
       </c>
       <c r="H153" s="20" t="inlineStr">
@@ -41072,7 +41072,7 @@
       </c>
       <c r="G154" s="20" t="inlineStr">
         <is>
-          <t>mensajeTecnicoProrroga</t>
+          <t>qd_mensajeTecnicoProrroga</t>
         </is>
       </c>
       <c r="H154" s="20" t="inlineStr">
@@ -41146,7 +41146,7 @@
       </c>
       <c r="G155" s="20" t="inlineStr">
         <is>
-          <t>payloadProrroga</t>
+          <t>qd_payloadProrroga</t>
         </is>
       </c>
       <c r="H155" s="20" t="inlineStr">
@@ -41224,7 +41224,7 @@
       </c>
       <c r="G156" s="20" t="inlineStr">
         <is>
-          <t>intentoProrroga</t>
+          <t>qd_intentoProrroga</t>
         </is>
       </c>
       <c r="H156" s="20" t="inlineStr">
@@ -41298,7 +41298,7 @@
       </c>
       <c r="G157" s="20" t="inlineStr">
         <is>
-          <t>causaRaizProrroga</t>
+          <t>qd_causaRaizProrroga</t>
         </is>
       </c>
       <c r="H157" s="20" t="inlineStr">
@@ -41372,7 +41372,7 @@
       </c>
       <c r="G158" s="20" t="inlineStr">
         <is>
-          <t>correccionProrroga</t>
+          <t>qd_correccionProrroga</t>
         </is>
       </c>
       <c r="H158" s="20" t="inlineStr">
@@ -41446,7 +41446,7 @@
       </c>
       <c r="G159" s="20" t="inlineStr">
         <is>
-          <t>codigoErrorProrroga</t>
+          <t>qd_codigoErrorProrroga</t>
         </is>
       </c>
       <c r="H159" s="20" t="inlineStr">
@@ -41520,7 +41520,7 @@
       </c>
       <c r="G160" s="20" t="inlineStr">
         <is>
-          <t>campoAfectadoProrroga</t>
+          <t>qd_campoAfectadoProrroga</t>
         </is>
       </c>
       <c r="H160" s="20" t="inlineStr">
@@ -41594,7 +41594,7 @@
       </c>
       <c r="G161" s="20" t="inlineStr">
         <is>
-          <t>mensajeErrorProrroga</t>
+          <t>qd_mensajeErrorProrroga</t>
         </is>
       </c>
       <c r="H161" s="20" t="inlineStr">
@@ -41668,7 +41668,7 @@
       </c>
       <c r="G162" s="20" t="inlineStr">
         <is>
-          <t>intentoActualProrroga</t>
+          <t>qd_intentoActualProrroga</t>
         </is>
       </c>
       <c r="H162" s="20" t="inlineStr">
@@ -41742,7 +41742,7 @@
       </c>
       <c r="G163" s="20" t="inlineStr">
         <is>
-          <t>motivoProrroga</t>
+          <t>qd_motivoProrroga</t>
         </is>
       </c>
       <c r="H163" s="20" t="inlineStr">
@@ -41824,7 +41824,7 @@
       </c>
       <c r="G164" s="20" t="inlineStr">
         <is>
-          <t>nuevaFechaLimite</t>
+          <t>qd_nuevaFechaLimite</t>
         </is>
       </c>
       <c r="H164" s="20" t="inlineStr">
@@ -41902,7 +41902,7 @@
       </c>
       <c r="G165" s="20" t="inlineStr">
         <is>
-          <t>contadorProrroga</t>
+          <t>qd_contadorProrroga</t>
         </is>
       </c>
       <c r="H165" s="20" t="inlineStr">
@@ -41980,7 +41980,7 @@
       </c>
       <c r="G166" s="20" t="inlineStr">
         <is>
-          <t>justificacionProrroga</t>
+          <t>qd_justificacionProrroga</t>
         </is>
       </c>
       <c r="H166" s="20" t="inlineStr">
@@ -42056,7 +42056,7 @@
       </c>
       <c r="G167" s="20" t="inlineStr">
         <is>
-          <t>idCasoBPM</t>
+          <t>qd_idCasoBPM</t>
         </is>
       </c>
       <c r="H167" s="20" t="inlineStr">
@@ -42132,7 +42132,7 @@
       </c>
       <c r="G168" s="20" t="inlineStr">
         <is>
-          <t>fechaCreacion</t>
+          <t>qd_fechaCreacion</t>
         </is>
       </c>
       <c r="H168" s="20" t="inlineStr">
@@ -42208,7 +42208,7 @@
       </c>
       <c r="G169" s="20" t="inlineStr">
         <is>
-          <t>tipoSolicitud</t>
+          <t>qd_tipoSolicitud</t>
         </is>
       </c>
       <c r="H169" s="20" t="inlineStr">
@@ -42288,7 +42288,7 @@
       </c>
       <c r="G170" s="20" t="inlineStr">
         <is>
-          <t>rolRadicador</t>
+          <t>qd_rolRadicador</t>
         </is>
       </c>
       <c r="H170" s="20" t="inlineStr">
@@ -42368,7 +42368,7 @@
       </c>
       <c r="G171" s="20" t="inlineStr">
         <is>
-          <t>puntoRecepcion</t>
+          <t>qd_puntoRecepcion</t>
         </is>
       </c>
       <c r="H171" s="20" t="inlineStr">
@@ -42448,7 +42448,7 @@
       </c>
       <c r="G172" s="20" t="inlineStr">
         <is>
-          <t>instanciaRecepcion</t>
+          <t>qd_instanciaRecepcion</t>
         </is>
       </c>
       <c r="H172" s="20" t="inlineStr">
@@ -42528,7 +42528,7 @@
       </c>
       <c r="G173" s="20" t="inlineStr">
         <is>
-          <t>tipoIdentificacion</t>
+          <t>qd_tipoIdentificacion</t>
         </is>
       </c>
       <c r="H173" s="20" t="inlineStr">
@@ -42608,7 +42608,7 @@
       </c>
       <c r="G174" s="20" t="inlineStr">
         <is>
-          <t>numeroIdentificacion</t>
+          <t>qd_numeroIdentificacion</t>
         </is>
       </c>
       <c r="H174" s="20" t="inlineStr">
@@ -42684,7 +42684,7 @@
       </c>
       <c r="G175" s="20" t="inlineStr">
         <is>
-          <t>nombres</t>
+          <t>qd_nombres</t>
         </is>
       </c>
       <c r="H175" s="20" t="inlineStr">
@@ -42760,7 +42760,7 @@
       </c>
       <c r="G176" s="20" t="inlineStr">
         <is>
-          <t>apellidos</t>
+          <t>qd_apellidos</t>
         </is>
       </c>
       <c r="H176" s="20" t="inlineStr">
@@ -42836,7 +42836,7 @@
       </c>
       <c r="G177" s="20" t="inlineStr">
         <is>
-          <t>razonSocial</t>
+          <t>qd_razonSocial</t>
         </is>
       </c>
       <c r="H177" s="20" t="inlineStr">
@@ -42912,7 +42912,7 @@
       </c>
       <c r="G178" s="20" t="inlineStr">
         <is>
-          <t>nombresContacto</t>
+          <t>qd_nombresContacto</t>
         </is>
       </c>
       <c r="H178" s="20" t="inlineStr">
@@ -42988,7 +42988,7 @@
       </c>
       <c r="G179" s="20" t="inlineStr">
         <is>
-          <t>apellidosContacto</t>
+          <t>qd_apellidosContacto</t>
         </is>
       </c>
       <c r="H179" s="20" t="inlineStr">
@@ -43064,7 +43064,7 @@
       </c>
       <c r="G180" s="20" t="inlineStr">
         <is>
-          <t>telefono</t>
+          <t>qd_telefono</t>
         </is>
       </c>
       <c r="H180" s="20" t="inlineStr">
@@ -43140,7 +43140,7 @@
       </c>
       <c r="G181" s="20" t="inlineStr">
         <is>
-          <t>correoElectronico</t>
+          <t>qd_correoElectronico</t>
         </is>
       </c>
       <c r="H181" s="20" t="inlineStr">
@@ -43216,7 +43216,7 @@
       </c>
       <c r="G182" s="20" t="inlineStr">
         <is>
-          <t>tipoPersona</t>
+          <t>qd_tipoPersona</t>
         </is>
       </c>
       <c r="H182" s="20" t="inlineStr">
@@ -43296,7 +43296,7 @@
       </c>
       <c r="G183" s="20" t="inlineStr">
         <is>
-          <t>codigoPais</t>
+          <t>qd_codigoPais</t>
         </is>
       </c>
       <c r="H183" s="20" t="inlineStr">
@@ -43376,7 +43376,7 @@
       </c>
       <c r="G184" s="20" t="inlineStr">
         <is>
-          <t>departamento</t>
+          <t>qd_departamento</t>
         </is>
       </c>
       <c r="H184" s="20" t="inlineStr">
@@ -43456,7 +43456,7 @@
       </c>
       <c r="G185" s="20" t="inlineStr">
         <is>
-          <t>municipio</t>
+          <t>qd_municipio</t>
         </is>
       </c>
       <c r="H185" s="20" t="inlineStr">
@@ -43536,7 +43536,7 @@
       </c>
       <c r="G186" s="20" t="inlineStr">
         <is>
-          <t>direccion</t>
+          <t>qd_direccion</t>
         </is>
       </c>
       <c r="H186" s="20" t="inlineStr">
@@ -43612,7 +43612,7 @@
       </c>
       <c r="G187" s="20" t="inlineStr">
         <is>
-          <t>sexo</t>
+          <t>qd_sexo</t>
         </is>
       </c>
       <c r="H187" s="20" t="inlineStr">
@@ -43692,7 +43692,7 @@
       </c>
       <c r="G188" s="20" t="inlineStr">
         <is>
-          <t>lgbtiq</t>
+          <t>qd_lgbtiq</t>
         </is>
       </c>
       <c r="H188" s="20" t="inlineStr">
@@ -43772,7 +43772,7 @@
       </c>
       <c r="G189" s="20" t="inlineStr">
         <is>
-          <t>condicionEspecial</t>
+          <t>qd_condicionEspecial</t>
         </is>
       </c>
       <c r="H189" s="20" t="inlineStr">
@@ -43852,7 +43852,7 @@
       </c>
       <c r="G190" s="20" t="inlineStr">
         <is>
-          <t>productoSFC</t>
+          <t>qd_productoSFC</t>
         </is>
       </c>
       <c r="H190" s="20" t="inlineStr">
@@ -43932,7 +43932,7 @@
       </c>
       <c r="G191" s="20" t="inlineStr">
         <is>
-          <t>detalleProducto</t>
+          <t>qd_detalleProducto</t>
         </is>
       </c>
       <c r="H191" s="20" t="inlineStr">
@@ -44012,7 +44012,7 @@
       </c>
       <c r="G192" s="20" t="inlineStr">
         <is>
-          <t>replica</t>
+          <t>qd_replica</t>
         </is>
       </c>
       <c r="H192" s="20" t="inlineStr">
@@ -44088,7 +44088,7 @@
       </c>
       <c r="G193" s="20" t="inlineStr">
         <is>
-          <t>argumentoReplica</t>
+          <t>qd_argumentoReplica</t>
         </is>
       </c>
       <c r="H193" s="20" t="inlineStr">
@@ -44164,7 +44164,7 @@
       </c>
       <c r="G194" s="20" t="inlineStr">
         <is>
-          <t>escalamientoDefensor</t>
+          <t>qd_escalamientoDefensor</t>
         </is>
       </c>
       <c r="H194" s="20" t="inlineStr">
@@ -44240,7 +44240,7 @@
       </c>
       <c r="G195" s="20" t="inlineStr">
         <is>
-          <t>motivoSFC</t>
+          <t>qd_motivoSFC</t>
         </is>
       </c>
       <c r="H195" s="20" t="inlineStr">
@@ -44320,7 +44320,7 @@
       </c>
       <c r="G196" s="20" t="inlineStr">
         <is>
-          <t>textoQueja</t>
+          <t>qd_textoQueja</t>
         </is>
       </c>
       <c r="H196" s="20" t="inlineStr">
@@ -44396,7 +44396,7 @@
       </c>
       <c r="G197" s="20" t="inlineStr">
         <is>
-          <t>anexos</t>
+          <t>qd_anexos</t>
         </is>
       </c>
       <c r="H197" s="20" t="inlineStr">
@@ -44472,7 +44472,7 @@
       </c>
       <c r="G198" s="20" t="inlineStr">
         <is>
-          <t>admision</t>
+          <t>qd_admision</t>
         </is>
       </c>
       <c r="H198" s="20" t="inlineStr">
@@ -44552,7 +44552,7 @@
       </c>
       <c r="G199" s="20" t="inlineStr">
         <is>
-          <t>enteControl</t>
+          <t>qd_enteControl</t>
         </is>
       </c>
       <c r="H199" s="20" t="inlineStr">
@@ -44632,7 +44632,7 @@
       </c>
       <c r="G200" s="20" t="inlineStr">
         <is>
-          <t>tutela</t>
+          <t>qd_tutela</t>
         </is>
       </c>
       <c r="H200" s="20" t="inlineStr">
@@ -44712,7 +44712,7 @@
       </c>
       <c r="G201" s="20" t="inlineStr">
         <is>
-          <t>quejaExpres</t>
+          <t>qd_quejaExpres</t>
         </is>
       </c>
       <c r="H201" s="20" t="inlineStr">
@@ -44792,7 +44792,7 @@
       </c>
       <c r="G202" s="20" t="inlineStr">
         <is>
-          <t>autorizacionDatos</t>
+          <t>qd_autorizacionDatos</t>
         </is>
       </c>
       <c r="H202" s="20" t="inlineStr">
@@ -44868,7 +44868,7 @@
       </c>
       <c r="G203" s="20" t="inlineStr">
         <is>
-          <t>captcha</t>
+          <t>qd_captcha</t>
         </is>
       </c>
       <c r="H203" s="20" t="inlineStr">
@@ -44944,7 +44944,7 @@
       </c>
       <c r="G204" s="20" t="inlineStr">
         <is>
-          <t>correoCopia</t>
+          <t>qd_correoCopia</t>
         </is>
       </c>
       <c r="H204" s="20" t="inlineStr">
@@ -45020,7 +45020,7 @@
       </c>
       <c r="G205" s="20" t="inlineStr">
         <is>
-          <t>estadoSmartSupervision</t>
+          <t>qd_estadoSmartSupervision</t>
         </is>
       </c>
       <c r="H205" s="20" t="inlineStr">
@@ -45096,7 +45096,7 @@
       </c>
       <c r="G206" s="20" t="inlineStr">
         <is>
-          <t>fechaRadicacionSFC</t>
+          <t>qd_fechaRadicacionSFC</t>
         </is>
       </c>
       <c r="H206" s="20" t="inlineStr">
@@ -45172,7 +45172,7 @@
       </c>
       <c r="G207" s="20" t="inlineStr">
         <is>
-          <t>rolResponsable</t>
+          <t>qd_rolResponsable</t>
         </is>
       </c>
       <c r="H207" s="20" t="inlineStr">
@@ -45248,7 +45248,7 @@
       </c>
       <c r="G208" s="20" t="inlineStr">
         <is>
-          <t>responsable</t>
+          <t>qd_responsable</t>
         </is>
       </c>
       <c r="H208" s="20" t="inlineStr">
@@ -45324,7 +45324,7 @@
       </c>
       <c r="G209" s="20" t="inlineStr">
         <is>
-          <t>nombreConsumidor</t>
+          <t>qd_nombres + qd_apellidos / qd_razonSocial</t>
         </is>
       </c>
       <c r="H209" s="20" t="inlineStr">
@@ -45400,7 +45400,7 @@
       </c>
       <c r="G210" s="20" t="inlineStr">
         <is>
-          <t>identificacion</t>
+          <t>qd_tipoIdentificacion + qd_numeroIdentificacion</t>
         </is>
       </c>
       <c r="H210" s="20" t="inlineStr">
@@ -45476,7 +45476,7 @@
       </c>
       <c r="G211" s="20" t="inlineStr">
         <is>
-          <t>correoElectronico</t>
+          <t>qd_correoElectronico</t>
         </is>
       </c>
       <c r="H211" s="20" t="inlineStr">
@@ -45552,7 +45552,7 @@
       </c>
       <c r="G212" s="20" t="inlineStr">
         <is>
-          <t>tipoPersona</t>
+          <t>qd_tipoPersona</t>
         </is>
       </c>
       <c r="H212" s="20" t="inlineStr">
@@ -45628,7 +45628,7 @@
       </c>
       <c r="G213" s="20" t="inlineStr">
         <is>
-          <t>canal</t>
+          <t>qd_canal</t>
         </is>
       </c>
       <c r="H213" s="20" t="inlineStr">
@@ -45704,7 +45704,7 @@
       </c>
       <c r="G214" s="20" t="inlineStr">
         <is>
-          <t>productoSFC</t>
+          <t>qd_productoSFC</t>
         </is>
       </c>
       <c r="H214" s="20" t="inlineStr">
@@ -45780,7 +45780,7 @@
       </c>
       <c r="G215" s="20" t="inlineStr">
         <is>
-          <t>motivoSFC</t>
+          <t>qd_motivoSFC</t>
         </is>
       </c>
       <c r="H215" s="20" t="inlineStr">
@@ -45856,7 +45856,7 @@
       </c>
       <c r="G216" s="20" t="inlineStr">
         <is>
-          <t>instanciaPunto</t>
+          <t>qd_instanciaRecepcion</t>
         </is>
       </c>
       <c r="H216" s="20" t="inlineStr">
@@ -45932,7 +45932,7 @@
       </c>
       <c r="G217" s="20" t="inlineStr">
         <is>
-          <t>admision</t>
+          <t>qd_admision</t>
         </is>
       </c>
       <c r="H217" s="20" t="inlineStr">
@@ -46008,7 +46008,7 @@
       </c>
       <c r="G218" s="20" t="inlineStr">
         <is>
-          <t>enteControl</t>
+          <t>qd_enteControl</t>
         </is>
       </c>
       <c r="H218" s="20" t="inlineStr">
@@ -46084,7 +46084,7 @@
       </c>
       <c r="G219" s="20" t="inlineStr">
         <is>
-          <t>resumen</t>
+          <t>qd_motivoSFC</t>
         </is>
       </c>
       <c r="H219" s="20" t="inlineStr">
@@ -46160,7 +46160,7 @@
       </c>
       <c r="G220" s="20" t="inlineStr">
         <is>
-          <t>textoQueja</t>
+          <t>qd_textoQueja</t>
         </is>
       </c>
       <c r="H220" s="20" t="inlineStr">
@@ -46236,7 +46236,7 @@
       </c>
       <c r="G221" s="20" t="inlineStr">
         <is>
-          <t>estadoSS</t>
+          <t>qd_estadoSS</t>
         </is>
       </c>
       <c r="H221" s="20" t="inlineStr">
@@ -46312,7 +46312,7 @@
       </c>
       <c r="G222" s="20" t="inlineStr">
         <is>
-          <t>intentosM1M2</t>
+          <t>qd_intentosM1M2</t>
         </is>
       </c>
       <c r="H222" s="20" t="inlineStr">
@@ -46388,7 +46388,7 @@
       </c>
       <c r="G223" s="20" t="inlineStr">
         <is>
-          <t>fechaRadicacion</t>
+          <t>qd_fechaRadicacion</t>
         </is>
       </c>
       <c r="H223" s="20" t="inlineStr">
@@ -46464,7 +46464,7 @@
       </c>
       <c r="G224" s="20" t="inlineStr">
         <is>
-          <t>areaResponsable</t>
+          <t>qd_areaResponsable</t>
         </is>
       </c>
       <c r="H224" s="20" t="inlineStr">
@@ -46544,7 +46544,7 @@
       </c>
       <c r="G225" s="20" t="inlineStr">
         <is>
-          <t>usuarioResponsable</t>
+          <t>qd_usuarioResponsable</t>
         </is>
       </c>
       <c r="H225" s="20" t="inlineStr">
@@ -46624,7 +46624,7 @@
       </c>
       <c r="G226" s="20" t="inlineStr">
         <is>
-          <t>observacionesAsignacion</t>
+          <t>qd_observacionesAsignacion</t>
         </is>
       </c>
       <c r="H226" s="20" t="inlineStr">
@@ -46700,7 +46700,7 @@
       </c>
       <c r="G227" s="20" t="inlineStr">
         <is>
-          <t>responsableActual</t>
+          <t>qd_responsableActual</t>
         </is>
       </c>
       <c r="H227" s="20" t="inlineStr">
@@ -46776,7 +46776,7 @@
       </c>
       <c r="G228" s="20" t="inlineStr">
         <is>
-          <t>areaDestino</t>
+          <t>qd_areaDestino</t>
         </is>
       </c>
       <c r="H228" s="20" t="inlineStr">
@@ -46856,7 +46856,7 @@
       </c>
       <c r="G229" s="20" t="inlineStr">
         <is>
-          <t>nuevoResponsable</t>
+          <t>qd_nuevoResponsable</t>
         </is>
       </c>
       <c r="H229" s="20" t="inlineStr">
@@ -46936,7 +46936,7 @@
       </c>
       <c r="G230" s="20" t="inlineStr">
         <is>
-          <t>motivoReasignacion</t>
+          <t>qd_motivoReasignacion</t>
         </is>
       </c>
       <c r="H230" s="20" t="inlineStr">
@@ -47016,7 +47016,7 @@
       </c>
       <c r="G231" s="20" t="inlineStr">
         <is>
-          <t>observacionesReasignacion</t>
+          <t>qd_observacionesReasignacion</t>
         </is>
       </c>
       <c r="H231" s="20" t="inlineStr">
@@ -47092,7 +47092,7 @@
       </c>
       <c r="G232" s="20" t="inlineStr">
         <is>
-          <t>historialAsignaciones</t>
+          <t>qd_historialAsignaciones</t>
         </is>
       </c>
       <c r="H232" s="20" t="inlineStr">
@@ -47168,7 +47168,7 @@
       </c>
       <c r="G233" s="20" t="inlineStr">
         <is>
-          <t>respuestaCliente</t>
+          <t>qd_respuestaCliente</t>
         </is>
       </c>
       <c r="H233" s="20" t="inlineStr">
@@ -47244,7 +47244,7 @@
       </c>
       <c r="G234" s="20" t="inlineStr">
         <is>
-          <t>accionesTomadas</t>
+          <t>qd_accionesTomadas</t>
         </is>
       </c>
       <c r="H234" s="20" t="inlineStr">
@@ -47320,7 +47320,7 @@
       </c>
       <c r="G235" s="20" t="inlineStr">
         <is>
-          <t>reconocimiento</t>
+          <t>qd_reconocimiento</t>
         </is>
       </c>
       <c r="H235" s="20" t="inlineStr">
@@ -47396,7 +47396,7 @@
       </c>
       <c r="G236" s="20" t="inlineStr">
         <is>
-          <t>adjuntosSoporte</t>
+          <t>qd_adjuntosSoporte</t>
         </is>
       </c>
       <c r="H236" s="20" t="inlineStr">
@@ -47472,7 +47472,7 @@
       </c>
       <c r="G237" s="20" t="inlineStr">
         <is>
-          <t>respuestaFavorDe</t>
+          <t>qd_respuestaFavorDe</t>
         </is>
       </c>
       <c r="H237" s="20" t="inlineStr">
@@ -47552,7 +47552,7 @@
       </c>
       <c r="G238" s="20" t="inlineStr">
         <is>
-          <t>areaResponsable</t>
+          <t>qd_areaResponsable</t>
         </is>
       </c>
       <c r="H238" s="20" t="inlineStr">
@@ -47628,7 +47628,7 @@
       </c>
       <c r="G239" s="20" t="inlineStr">
         <is>
-          <t>usuarioResponsable</t>
+          <t>qd_usuarioResponsable</t>
         </is>
       </c>
       <c r="H239" s="20" t="inlineStr">
@@ -47704,7 +47704,7 @@
       </c>
       <c r="G240" s="20" t="inlineStr">
         <is>
-          <t>observacionesAsignacion</t>
+          <t>qd_observacionesAsignacion</t>
         </is>
       </c>
       <c r="H240" s="20" t="inlineStr">
@@ -47780,7 +47780,7 @@
       </c>
       <c r="G241" s="20" t="inlineStr">
         <is>
-          <t>comentarioArea</t>
+          <t>qd_comentarioArea</t>
         </is>
       </c>
       <c r="H241" s="20" t="inlineStr">
@@ -47856,7 +47856,7 @@
       </c>
       <c r="G242" s="20" t="inlineStr">
         <is>
-          <t>adjuntoArea</t>
+          <t>qd_adjuntoArea</t>
         </is>
       </c>
       <c r="H242" s="20" t="inlineStr">
@@ -47932,7 +47932,7 @@
       </c>
       <c r="G243" s="20" t="inlineStr">
         <is>
-          <t>nombreConsumidor</t>
+          <t>qd_nombres + qd_apellidos / qd_razonSocial</t>
         </is>
       </c>
       <c r="H243" s="20" t="inlineStr">
@@ -48008,7 +48008,7 @@
       </c>
       <c r="G244" s="20" t="inlineStr">
         <is>
-          <t>identificacion</t>
+          <t>qd_tipoIdentificacion + qd_numeroIdentificacion</t>
         </is>
       </c>
       <c r="H244" s="20" t="inlineStr">
@@ -48084,7 +48084,7 @@
       </c>
       <c r="G245" s="20" t="inlineStr">
         <is>
-          <t>correoElectronico</t>
+          <t>qd_correoElectronico</t>
         </is>
       </c>
       <c r="H245" s="20" t="inlineStr">
@@ -48160,7 +48160,7 @@
       </c>
       <c r="G246" s="20" t="inlineStr">
         <is>
-          <t>tipoPersona</t>
+          <t>qd_tipoPersona</t>
         </is>
       </c>
       <c r="H246" s="20" t="inlineStr">
@@ -48236,7 +48236,7 @@
       </c>
       <c r="G247" s="20" t="inlineStr">
         <is>
-          <t>canal</t>
+          <t>qd_canal</t>
         </is>
       </c>
       <c r="H247" s="20" t="inlineStr">
@@ -48312,7 +48312,7 @@
       </c>
       <c r="G248" s="20" t="inlineStr">
         <is>
-          <t>productoSFC</t>
+          <t>qd_productoSFC</t>
         </is>
       </c>
       <c r="H248" s="20" t="inlineStr">
@@ -48388,7 +48388,7 @@
       </c>
       <c r="G249" s="20" t="inlineStr">
         <is>
-          <t>motivoSFC</t>
+          <t>qd_motivoSFC</t>
         </is>
       </c>
       <c r="H249" s="20" t="inlineStr">
@@ -48464,7 +48464,7 @@
       </c>
       <c r="G250" s="20" t="inlineStr">
         <is>
-          <t>instanciaPunto</t>
+          <t>qd_instanciaRecepcion</t>
         </is>
       </c>
       <c r="H250" s="20" t="inlineStr">
@@ -48540,7 +48540,7 @@
       </c>
       <c r="G251" s="20" t="inlineStr">
         <is>
-          <t>admision</t>
+          <t>qd_admision</t>
         </is>
       </c>
       <c r="H251" s="20" t="inlineStr">
@@ -48616,7 +48616,7 @@
       </c>
       <c r="G252" s="20" t="inlineStr">
         <is>
-          <t>enteControl</t>
+          <t>qd_enteControl</t>
         </is>
       </c>
       <c r="H252" s="20" t="inlineStr">
@@ -48692,7 +48692,7 @@
       </c>
       <c r="G253" s="20" t="inlineStr">
         <is>
-          <t>resumen</t>
+          <t>qd_motivoSFC</t>
         </is>
       </c>
       <c r="H253" s="20" t="inlineStr">
@@ -48768,7 +48768,7 @@
       </c>
       <c r="G254" s="20" t="inlineStr">
         <is>
-          <t>textoQueja</t>
+          <t>qd_textoQueja</t>
         </is>
       </c>
       <c r="H254" s="20" t="inlineStr">
@@ -48834,7 +48834,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I51"/>
+  <dimension ref="B1:I51"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="14.45"/>
   <cols>
     <col width="3" customWidth="1" style="105" min="1" max="1"/>
@@ -51019,7 +51019,7 @@
       </c>
       <c r="G7" s="37" t="inlineStr">
         <is>
-          <t>numeroIdentificacion contiene letras o longitud &lt;6 o &gt;15</t>
+          <t>qd_numeroIdentificacion contiene letras o longitud &lt;6 o &gt;15</t>
         </is>
       </c>
       <c r="H7" s="37" t="inlineStr">
@@ -51133,7 +51133,7 @@
       </c>
       <c r="G9" s="37" t="inlineStr">
         <is>
-          <t>resumen o nombreConsumidor contienen caracteres no permitidos SFC</t>
+          <t>qd_nombres, qd_apellidos o qd_razonSocial contienen caracteres no permitidos SFC</t>
         </is>
       </c>
       <c r="H9" s="37" t="inlineStr">
@@ -53014,7 +53014,7 @@
       </c>
       <c r="G42" s="37" t="inlineStr">
         <is>
-          <t>textoQueja tiene menos de 50 o más de 2000 caracteres</t>
+          <t>qd_textoQueja tiene menos de 50 o más de 2000 caracteres</t>
         </is>
       </c>
       <c r="H42" s="37" t="inlineStr">
@@ -53413,7 +53413,7 @@
       </c>
       <c r="G49" s="37" t="inlineStr">
         <is>
-          <t>numeroIdentificacion no cumple el formato según el tipo de documento</t>
+          <t>qd_numeroIdentificacion no cumple el formato según el tipo de documento</t>
         </is>
       </c>
       <c r="H49" s="37" t="inlineStr">

</xml_diff>